<commit_message>
Added the PED.md file and Decision log cascaded updates
Updated the decision log , constraints, stakeholder register and conflict register to match with additional constraints. Also added section 2 of the PED document for review
</commit_message>
<xml_diff>
--- a/docs/Requirements/Constraints.xlsx
+++ b/docs/Requirements/Constraints.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c906530d9ff38bc/Desktop/SEN381/Ticketing-System/docs/Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4A4B3C61-DD64-4070-BD95-BDFD6A0DE2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="8_{4A4B3C61-DD64-4070-BD95-BDFD6A0DE2B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59E8B72F-08EE-4781-8956-3FD6F7C3D5C8}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{B629CCF1-2F03-4A13-AACC-A7A6BED89A4B}"/>
+    <workbookView xWindow="9228" yWindow="0" windowWidth="21588" windowHeight="17376" xr2:uid="{B629CCF1-2F03-4A13-AACC-A7A6BED89A4B}"/>
   </bookViews>
   <sheets>
     <sheet name="Constraints" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="116">
   <si>
     <t>Constraints</t>
   </si>
@@ -216,13 +216,184 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>CON-009</t>
+  </si>
+  <si>
+    <t>CON-010</t>
+  </si>
+  <si>
+    <t>CON-011</t>
+  </si>
+  <si>
+    <t>CON-012</t>
+  </si>
+  <si>
+    <t>CON-013</t>
+  </si>
+  <si>
+    <t>Effort and development time must be estimated (COCOMO / PERT)</t>
+  </si>
+  <si>
+    <t>Lecturer instruction, verbal, week of 09/09/2026 — recorded in team notes</t>
+  </si>
+  <si>
+    <t>Verbally ; STK-010</t>
+  </si>
+  <si>
+    <t>Requires a size estimate before M2 scope can be responsibly fixed. A three-student team on a well-understood problem falls in COCOMO Organic mode (a=2.4, b=1.05), so the estimate is only as good as the size input. If the calculated development time exceeds the available delivery period, scope must be reduced rather than the estimate optimistically adjusted.</t>
+  </si>
+  <si>
+    <t>CON-002, CON-001, DEC-002</t>
+  </si>
+  <si>
+    <t>COCOMO takes kLOC as input, but lines of code vary by an order of magnitude across stacks — and DEC-002 defers stack selection. Either produce the estimate against a documented assumed stack and revise it after M2, or delay the estimate and lose its value as a scope check. We take the first option and record the assumption.</t>
+  </si>
+  <si>
+    <t>The system must support approximately 100 users, with the team able to reason about behaviour at 1000</t>
+  </si>
+  <si>
+    <t>Converts a vague scalability aspiration into a testable figure for Member B's NFRs. 100 concurrent users is modest, but the tenfold headroom rules out designs dependent on in-memory session state or unindexed table scans. Drives indexing strategy, connection pooling and query design in M2, and is verifiable under CON-005 in M3.</t>
+  </si>
+  <si>
+    <t>CON-003, CON-005</t>
+  </si>
+  <si>
+    <t>Free-tier platforms commonly cap concurrent connections and database compute. The 1000-user headroom may exceed what the cost constraint permits, which feeds directly into the deferred hosting decision (DEC-003).</t>
+  </si>
+  <si>
+    <t>The solution must be delivered as a web application; mobile access is provided through responsive web rather than a native application</t>
+  </si>
+  <si>
+    <t>Confirms the exclusion already recorded in SCP-013 and DEC-007, but changes its status from team judgement to client directive — it can no longer be revisited without a change request. Places a responsive-design obligation on the interface and creates a mobile-viewport quality attribute that must be specified measurably.</t>
+  </si>
+  <si>
+    <t>CON-001, DEC-007</t>
+  </si>
+  <si>
+    <t>Responsive web avoids a second build and release path, but limits access to device capabilities. If photograph attachments (SCP-015) are reinstated, capture will depend on browser file APIs rather than native camera access.</t>
+  </si>
+  <si>
+    <t>The solution must implement a layered architecture</t>
+  </si>
+  <si>
+    <t>Removes architectural style from the M2 decision space. The M2 ADR therefore records rationale, layer boundaries and dependency rules rather than selecting between styles. Enforces that presentation code does not reach data access directly, which improves testability under CON-005 but adds mapping code between layers.</t>
+  </si>
+  <si>
+    <t>CON-004, CON-005</t>
+  </si>
+  <si>
+    <t>A prescribed style may not be optimal for the problem, but it lowers risk and learning curve for a team of three (CON-004). The team must still justify where the layer boundaries fall — that judgement remains ours and remains assessable.</t>
+  </si>
+  <si>
+    <t>Demonstrable progress on frontend, backend and APIs is required from week 3 of the delivery period</t>
+  </si>
+  <si>
+    <t>Overlaps construction with the M2 design phase rather than following it. Forces a technology commitment earlier than the evidence-gathering in DEC-002 and DEC-003 anticipated, and raises the risk of building against requirements that are not yet stable.</t>
+  </si>
+  <si>
+    <t>CON-002, DEC-002, DEC-003</t>
+  </si>
+  <si>
+    <t>Early construction produces feedback and reduces late integration risk, but compresses the window for platform and stack evaluation. The correct response is to record the acceleration and its risk rather than to claim the M1?M2?M3 sequence held unchanged.</t>
+  </si>
+  <si>
+    <t>CON-014</t>
+  </si>
+  <si>
+    <t>CON-015</t>
+  </si>
+  <si>
+    <t>CON-016</t>
+  </si>
+  <si>
+    <t>CON-017</t>
+  </si>
+  <si>
+    <t>CON-018</t>
+  </si>
+  <si>
+    <t>CON-019</t>
+  </si>
+  <si>
+    <t>The system must produce logging sufficient to observe and check runtime performance</t>
+  </si>
+  <si>
+    <t>Performance cannot be claimed under CON-005 without measurement, and measurement cannot be retrofitted after an incident. Logging must be designed alongside the architecture in M2, not added in M3. Also supplies the evidence needed to verify the response-time and capacity figures in CON-010.</t>
+  </si>
+  <si>
+    <t>CON-005, CON-007, CON-010</t>
+  </si>
+  <si>
+    <t>Performance logs that include request context risk capturing personal information, which CON-007 restricts. Log content and retention must be designed deliberately rather than defaulted.</t>
+  </si>
+  <si>
+    <t>Database changes must be version controlled and auditable via triggers and logging</t>
+  </si>
+  <si>
+    <t>Extends configuration control from source code to database state, matching the requirement that DB scripts be identifiable, versioned and controlled. Trigger-based audit also supplies the attribution needed for SCP-008 (recorded acting user) and the accountability the scenario identifies as missing.</t>
+  </si>
+  <si>
+    <t>CON-006, CON-007, CON-010</t>
+  </si>
+  <si>
+    <t>Triggers move audit logic into the database where it cannot be bypassed by the application, but they are harder to test and version than application-level auditing, and they add write overhead that matters at the CON-010 capacity figure.</t>
+  </si>
+  <si>
+    <t>Development, test, staging and production must use separate database schemas</t>
+  </si>
+  <si>
+    <t>Requires environment-specific configuration to be controlled from M2 rather than improvised at deployment, and makes schema migration a repeatable, scripted process rather than a manual one. Also prevents test data from reaching production data under CON-007.</t>
+  </si>
+  <si>
+    <t>CON-003, CON-006, CON-015</t>
+  </si>
+  <si>
+    <t>Multiple schemas may exceed free-tier database allowances, feeding the deferred hosting decision (DEC-003). Environment parity also becomes an obligation — divergence between staging and production undermines the value of having both.</t>
+  </si>
+  <si>
+    <t>Database operations must be transactional so that faulty transactions can be rolled back</t>
+  </si>
+  <si>
+    <t>Status transitions and assignment changes (SCP-007, SCP-008) touch multiple tables including the audit trail. Without transactional boundaries a partial failure leaves the lifecycle record inconsistent, which defeats the single-authoritative-record purpose in PED 2.2. Constrains the persistence choice in M2 toward a store with real transaction support.</t>
+  </si>
+  <si>
+    <t>CON-015, DEC-002</t>
+  </si>
+  <si>
+    <t>Transactional guarantees cost concurrency under load. At the CON-010 figure this is unlikely to bind, but the boundaries must be scoped deliberately rather than wrapping whole request handlers.</t>
+  </si>
+  <si>
+    <t>The database must use an appropriate indexing strategy</t>
+  </si>
+  <si>
+    <t>The search, filter and sort capability (SCP-006) and the management reporting views (SCP-011) are the queries that degrade first as volume grows. Indexing is what makes the CON-010 headroom achievable. Index selection must be justified against actual query patterns rather than added uniformly.</t>
+  </si>
+  <si>
+    <t>CON-010, CON-005</t>
+  </si>
+  <si>
+    <t>Indexes speed reads and slow writes. Combined with the trigger-based auditing in CON-015, write cost compounds — every status change writes the record, the audit row and every affected index.</t>
+  </si>
+  <si>
+    <t>The system must implement role-based access control, user grouping and appropriate encryption, and will be actively probed for weaknesses during assessment</t>
+  </si>
+  <si>
+    <t>Confirms and hardens CON-006 and SCP-012. The assessment method matters engineering-wise: controls will be tested adversarially, so authorisation must be enforced server-side at every entry point rather than by hiding interface elements. Encryption obligations apply in transit and at rest for the personal information under CON-007.</t>
+  </si>
+  <si>
+    <t>CON-006, CON-007, CON-003</t>
+  </si>
+  <si>
+    <t>Encryption at rest and managed identity are frequently paid features on otherwise-free platforms — another input to DEC-003. Server-side authorisation checks at every endpoint add development and test effort under CON-002.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -288,6 +459,12 @@
       <b/>
       <sz val="12"/>
       <color rgb="FF0F4761"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -383,8 +560,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -394,42 +622,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -439,94 +631,35 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFA61B1B"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFBE3E3"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF0F4761"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE4F1F8"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF1E6B2C"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFE2F0E4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF7A3E00"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFF3D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF4A2D80"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFEDE7F8"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <font>
         <b/>
@@ -922,7 +1055,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A8CAEAA-E1A8-43E2-A3CE-E0545A1AE5E4}">
-  <dimension ref="B1:L12"/>
+  <dimension ref="B1:L23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="2.21875" customWidth="1"/>
@@ -938,285 +1071,538 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:12" ht="25.8" x14ac:dyDescent="0.3">
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
     </row>
     <row r="2" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
     </row>
     <row r="4" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="K4" s="17"/>
-      <c r="L4" s="18"/>
-    </row>
-    <row r="5" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B5" s="6" t="s">
+      <c r="K4" s="22"/>
+      <c r="L4" s="23"/>
+    </row>
+    <row r="5" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="E5" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="H5" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="J5" s="19" t="s">
+      <c r="J5" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="K5" s="19"/>
-      <c r="L5" s="20">
-        <f>COUNTIF($C$5:$C$12,"Scope")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="11" t="s">
+      <c r="K5" s="16"/>
+      <c r="L5" s="12">
+        <f>COUNTIF($C$5:$C$58,"Scope")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B6" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="24" t="s">
+      <c r="F6" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="13" t="s">
+      <c r="H6" s="30" t="s">
         <v>21</v>
       </c>
-      <c r="J6" s="19" t="s">
+      <c r="J6" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="19"/>
-      <c r="L6" s="20">
-        <f>COUNTIF($C$5:$C$12,"Schedule")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B7" s="6" t="s">
+      <c r="K6" s="16"/>
+      <c r="L6" s="12">
+        <f>COUNTIF($C$5:$C$65,"Schedule")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="D7" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="8" t="s">
+      <c r="H7" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="19" t="s">
+      <c r="J7" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="19"/>
-      <c r="L7" s="20">
-        <f>COUNTIF($C$5:$C$12,"Cost &amp; resources")</f>
+      <c r="K7" s="16"/>
+      <c r="L7" s="12">
+        <f>COUNTIF($C$5:$C$58,"Cost &amp; resources")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="11" t="s">
+    <row r="8" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="E8" s="14" t="s">
+      <c r="E8" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="24" t="s">
+      <c r="F8" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="G8" s="15" t="s">
+      <c r="G8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="J8" s="19" t="s">
+      <c r="J8" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="K8" s="19"/>
-      <c r="L8" s="20">
-        <f>COUNTIF($C$5:$C$12,"Quality")</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B9" s="6" t="s">
+      <c r="K8" s="16"/>
+      <c r="L8" s="12">
+        <f>COUNTIF($C$5:$C$63,"Quality")</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B9" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="E9" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="J9" s="19" t="s">
+      <c r="J9" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="K9" s="19"/>
-      <c r="L9" s="20">
-        <f>COUNTIF($C$5:$C$12,"Security")</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B10" s="11" t="s">
+      <c r="K9" s="16"/>
+      <c r="L9" s="12">
+        <f>COUNTIF($C$5:$C$56,"Security")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B10" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="G10" s="15" t="s">
+      <c r="G10" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="13" t="s">
+      <c r="H10" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="J10" s="21" t="s">
+      <c r="J10" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="K10" s="21"/>
-      <c r="L10" s="22">
-        <f>COUNTA($B$5:$B$12)</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B11" s="6" t="s">
+      <c r="K10" s="17"/>
+      <c r="L10" s="13">
+        <f>COUNTA($B$5:$B$64)</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B11" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="E11" s="9" t="s">
+      <c r="E11" s="27" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="23" t="s">
+      <c r="F11" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="H11" s="8" t="s">
+      <c r="H11" s="26" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="12" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B12" s="11" t="s">
+    <row r="12" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B12" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="28" t="s">
         <v>53</v>
       </c>
-      <c r="F12" s="24" t="s">
+      <c r="F12" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="G12" s="15" t="s">
+      <c r="G12" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="30" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B13" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="H13" s="29" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B14" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="30" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="H14" s="30" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B15" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F15" s="31" t="s">
+        <v>75</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="H15" s="31" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B16" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="72" x14ac:dyDescent="0.3">
+      <c r="B17" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>82</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F17" s="31" t="s">
+        <v>83</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="H17" s="31" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B18" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="29" t="s">
+        <v>92</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F18" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H18" s="31" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B19" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C19" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F19" s="31" t="s">
+        <v>97</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H19" s="31" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B20" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C20" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D20" s="29" t="s">
+        <v>100</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F20" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="H20" s="31" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B21" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="29" t="s">
+        <v>104</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F21" s="31" t="s">
+        <v>105</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H21" s="31" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B22" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="D22" s="29" t="s">
+        <v>108</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>109</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="H22" s="31" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B23" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="29" t="s">
+        <v>112</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F23" s="31" t="s">
+        <v>113</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="H23" s="31" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1231,7 +1617,8 @@
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="J7:K7"/>
   </mergeCells>
-  <conditionalFormatting sqref="C5:C12">
+  <phoneticPr fontId="9" type="noConversion"/>
+  <conditionalFormatting sqref="C5:C23">
     <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Scope">
       <formula>NOT(ISERROR(SEARCH("Scope",C5)))</formula>
     </cfRule>

</xml_diff>